<commit_message>
Update 12626434.xlsx - 16 August 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -1024,7 +1024,60 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="28.8" customHeight="1"/>
+    <row r="8" ht="28.8" customHeight="1">
+      <c r="A8" s="13" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="E8" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="F8" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I8" s="15">
+        <f>IF(SUM(B8:F8,H8)=0,"",SUM(B8:F8,H8))</f>
+        <v/>
+      </c>
+      <c r="J8" s="15">
+        <f>IF(I8="","",1440-I8)</f>
+        <v/>
+      </c>
+      <c r="K8" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L8" s="16" t="inlineStr">
+        <is>
+          <t>Unsatisfied</t>
+        </is>
+      </c>
+      <c r="M8" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>No regular classes. Studied at home and relaxed.</t>
+        </is>
+      </c>
+    </row>
     <row r="9" ht="28.8" customHeight="1"/>
     <row r="10" ht="43.2" customHeight="1"/>
     <row r="11" ht="43.2" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 18 August 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -1078,8 +1078,116 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="28.8" customHeight="1"/>
-    <row r="10" ht="43.2" customHeight="1"/>
+    <row r="9" ht="28.8" customHeight="1">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 2026-08-17</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="14" t="n">
+        <v>240</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I9" s="15">
+        <f>IF(SUM(B9:F9,H9)=0,"",SUM(B9:F9,H9))</f>
+        <v/>
+      </c>
+      <c r="J9" s="15">
+        <f>IF(I9="","",1440-I9)</f>
+        <v/>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M9" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N9" s="17" t="inlineStr">
+        <is>
+          <t>No regular classes. Studied at home and relaxed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="43.2" customHeight="1">
+      <c r="A10" s="13" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B10" s="14" t="n">
+        <v>360</v>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D10" s="14" t="n">
+        <v>90</v>
+      </c>
+      <c r="E10" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F10" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G10" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H10" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="I10" s="15">
+        <f>IF(SUM(B10:F10,H10)=0,"",SUM(B10:F10,H10))</f>
+        <v/>
+      </c>
+      <c r="J10" s="15">
+        <f>IF(I10="","",1440-I10)</f>
+        <v/>
+      </c>
+      <c r="K10" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L10" s="16" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M10" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>Classes were a little tiring; did some revision after coming home.</t>
+        </is>
+      </c>
+    </row>
     <row r="11" ht="43.2" customHeight="1"/>
     <row r="12" ht="28.8" customHeight="1"/>
     <row r="13" ht="28.8" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 19 August 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -1188,7 +1188,60 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="43.2" customHeight="1"/>
+    <row r="11" ht="43.2" customHeight="1">
+      <c r="A11" s="13" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B11" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D11" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="F11" s="14" t="n">
+        <v>350</v>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="H11" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I11" s="15">
+        <f>IF(SUM(B11:F11,H11)=0,"",SUM(B11:F11,H11))</f>
+        <v/>
+      </c>
+      <c r="J11" s="15">
+        <f>IF(I11="","",1440-I11)</f>
+        <v/>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M11" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N11" s="17" t="inlineStr">
+        <is>
+          <t>Classes were a little tiring; did some revision after coming home.</t>
+        </is>
+      </c>
+    </row>
     <row r="12" ht="28.8" customHeight="1"/>
     <row r="13" ht="28.8" customHeight="1"/>
     <row r="14" ht="43.2" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 20 August 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -1242,7 +1242,60 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="28.8" customHeight="1"/>
+    <row r="12" ht="28.8" customHeight="1">
+      <c r="A12" s="13" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B12" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="D12" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H12" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="I12" s="15">
+        <f>IF(SUM(B12:F12,H12)=0,"",SUM(B12:F12,H12))</f>
+        <v/>
+      </c>
+      <c r="J12" s="15">
+        <f>IF(I12="","",1440-I12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L12" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M12" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>Had regular classes and completed a little study at night.</t>
+        </is>
+      </c>
+    </row>
     <row r="13" ht="28.8" customHeight="1"/>
     <row r="14" ht="43.2" customHeight="1"/>
     <row r="16" ht="28.8" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 21 August 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -1296,7 +1296,60 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="28.8" customHeight="1"/>
+    <row r="13" ht="28.8" customHeight="1">
+      <c r="A13" s="13" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B13" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C13" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="D13" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E13" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="F13" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G13" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H13" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="I13" s="15">
+        <f>IF(SUM(B13:F13,H13)=0,"",SUM(B13:F13,H13))</f>
+        <v/>
+      </c>
+      <c r="J13" s="15">
+        <f>IF(I13="","",1440-I13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M13" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N13" s="17" t="inlineStr">
+        <is>
+          <t>Had regular classes and completed a little study at night.</t>
+        </is>
+      </c>
+    </row>
     <row r="14" ht="43.2" customHeight="1"/>
     <row r="16" ht="28.8" customHeight="1"/>
     <row r="17" ht="28.8" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 22 August 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -1350,7 +1350,60 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="43.2" customHeight="1"/>
+    <row r="14" ht="43.2" customHeight="1">
+      <c r="A14" s="13" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B14" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C14" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I14" s="15">
+        <f>IF(SUM(B14:F14,H14)=0,"",SUM(B14:F14,H14))</f>
+        <v/>
+      </c>
+      <c r="J14" s="15">
+        <f>IF(I14="","",1440-I14)</f>
+        <v/>
+      </c>
+      <c r="K14" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L14" s="16" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M14" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>No regular classes. Studied at home watching movie and relaxed.</t>
+        </is>
+      </c>
+    </row>
     <row r="16" ht="28.8" customHeight="1"/>
     <row r="17" ht="28.8" customHeight="1"/>
     <row r="18" ht="28.8" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 23 August 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -1401,6 +1401,60 @@
       <c r="N14" s="17" t="inlineStr">
         <is>
           <t>No regular classes. Studied at home watching movie and relaxed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B15" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C15" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D15" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I15" s="15">
+        <f>IF(SUM(B15:F15,H15)=0,"",SUM(B15:F15,H15))</f>
+        <v/>
+      </c>
+      <c r="J15" s="15">
+        <f>IF(I15="","",1440-I15)</f>
+        <v/>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>Unsatisfied</t>
+        </is>
+      </c>
+      <c r="M15" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N15" s="17" t="inlineStr">
+        <is>
+          <t>Less study due to sickness.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 25 August 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -1512,7 +1512,60 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="28.8" customHeight="1"/>
+    <row r="17" ht="28.8" customHeight="1">
+      <c r="A17" s="13" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B17" s="14" t="n">
+        <v>360</v>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="F17" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H17" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="I17" s="15">
+        <f>IF(SUM(B17:F17,H17)=0,"",SUM(B17:F17,H17))</f>
+        <v/>
+      </c>
+      <c r="J17" s="15">
+        <f>IF(I17="","",1440-I17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M17" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N17" s="17" t="inlineStr">
+        <is>
+          <t>Had regular classes and completed a little study at night.</t>
+        </is>
+      </c>
+    </row>
     <row r="18" ht="28.8" customHeight="1"/>
     <row r="19" ht="28.8" customHeight="1"/>
     <row r="20" ht="28.8" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 26 August 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -1566,7 +1566,60 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="28.8" customHeight="1"/>
+    <row r="18" ht="28.8" customHeight="1">
+      <c r="A18" s="13" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B18" s="14" t="n">
+        <v>360</v>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="D18" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="F18" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H18" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="I18" s="15">
+        <f>IF(SUM(B18:F18,H18)=0,"",SUM(B18:F18,H18))</f>
+        <v/>
+      </c>
+      <c r="J18" s="15">
+        <f>IF(I18="","",1440-I18)</f>
+        <v/>
+      </c>
+      <c r="K18" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L18" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M18" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>Had regular classes and completed a little study at night.</t>
+        </is>
+      </c>
+    </row>
     <row r="19" ht="28.8" customHeight="1"/>
     <row r="20" ht="28.8" customHeight="1"/>
     <row r="21" ht="28.8" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 27 August 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -1620,7 +1620,60 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="28.8" customHeight="1"/>
+    <row r="19" ht="28.8" customHeight="1">
+      <c r="A19" s="13" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B19" s="14" t="n">
+        <v>360</v>
+      </c>
+      <c r="C19" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D19" s="14" t="n">
+        <v>90</v>
+      </c>
+      <c r="E19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="G19" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H19" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="I19" s="15">
+        <f>IF(SUM(B19:F19,H19)=0,"",SUM(B19:F19,H19))</f>
+        <v/>
+      </c>
+      <c r="J19" s="15">
+        <f>IF(I19="","",1440-I19)</f>
+        <v/>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M19" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N19" s="17" t="inlineStr">
+        <is>
+          <t>Completed daily tasks and some exercise.</t>
+        </is>
+      </c>
+    </row>
     <row r="20" ht="28.8" customHeight="1"/>
     <row r="21" ht="28.8" customHeight="1"/>
     <row r="22" ht="28.8" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 28 August 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -1674,7 +1674,60 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="28.8" customHeight="1"/>
+    <row r="20" ht="28.8" customHeight="1">
+      <c r="A20" s="13" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B20" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C20" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E20" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="G20" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H20" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I20" s="15">
+        <f>IF(SUM(B20:F20,H20)=0,"",SUM(B20:F20,H20))</f>
+        <v/>
+      </c>
+      <c r="J20" s="15">
+        <f>IF(I20="","",1440-I20)</f>
+        <v/>
+      </c>
+      <c r="K20" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L20" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M20" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>Had regular classes and completed a little study at night.</t>
+        </is>
+      </c>
+    </row>
     <row r="21" ht="28.8" customHeight="1"/>
     <row r="22" ht="28.8" customHeight="1"/>
     <row r="23" ht="28.8" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 29 August 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -1728,7 +1728,60 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="28.8" customHeight="1"/>
+    <row r="21" ht="28.8" customHeight="1">
+      <c r="A21" s="13" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B21" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C21" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D21" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="E21" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I21" s="15">
+        <f>IF(SUM(B21:F21,H21)=0,"",SUM(B21:F21,H21))</f>
+        <v/>
+      </c>
+      <c r="J21" s="15">
+        <f>IF(I21="","",1440-I21)</f>
+        <v/>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L21" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M21" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N21" s="17" t="inlineStr">
+        <is>
+          <t>No regular classes. Studied at home and relaxed.</t>
+        </is>
+      </c>
+    </row>
     <row r="22" ht="28.8" customHeight="1"/>
     <row r="23" ht="28.8" customHeight="1"/>
     <row r="24" ht="43.2" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 30 August 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -1782,7 +1782,60 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="28.8" customHeight="1"/>
+    <row r="22" ht="28.8" customHeight="1">
+      <c r="A22" s="13" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B22" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C22" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="D22" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="E22" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F22" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="I22" s="15">
+        <f>IF(SUM(B22:F22,H22)=0,"",SUM(B22:F22,H22))</f>
+        <v/>
+      </c>
+      <c r="J22" s="15">
+        <f>IF(I22="","",1440-I22)</f>
+        <v/>
+      </c>
+      <c r="K22" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L22" s="16" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M22" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N22" s="17" t="inlineStr">
+        <is>
+          <t>No regular classes. Studied at home and relaxed.</t>
+        </is>
+      </c>
+    </row>
     <row r="23" ht="28.8" customHeight="1"/>
     <row r="24" ht="43.2" customHeight="1"/>
     <row r="25" ht="43.2" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 31 August 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -1836,7 +1836,60 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="28.8" customHeight="1"/>
+    <row r="23" ht="28.8" customHeight="1">
+      <c r="A23" s="13" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B23" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C23" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D23" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E23" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="F23" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H23" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="I23" s="15">
+        <f>IF(SUM(B23:F23,H23)=0,"",SUM(B23:F23,H23))</f>
+        <v/>
+      </c>
+      <c r="J23" s="15">
+        <f>IF(I23="","",1440-I23)</f>
+        <v/>
+      </c>
+      <c r="K23" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L23" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M23" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N23" s="17" t="inlineStr">
+        <is>
+          <t>Had regular classes and completed a little study at night.</t>
+        </is>
+      </c>
+    </row>
     <row r="24" ht="43.2" customHeight="1"/>
     <row r="25" ht="43.2" customHeight="1"/>
     <row r="26" ht="28.8" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 01 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -1890,7 +1890,60 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="43.2" customHeight="1"/>
+    <row r="24" ht="43.2" customHeight="1">
+      <c r="A24" s="13" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B24" s="14" t="n">
+        <v>360</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D24" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="E24" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F24" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H24" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I24" s="15">
+        <f>IF(SUM(B24:F24,H24)=0,"",SUM(B24:F24,H24))</f>
+        <v/>
+      </c>
+      <c r="J24" s="15">
+        <f>IF(I24="","",1440-I24)</f>
+        <v/>
+      </c>
+      <c r="K24" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L24" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M24" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N24" s="17" t="inlineStr">
+        <is>
+          <t>Classes were a little tiring and did some revision after coming home.</t>
+        </is>
+      </c>
+    </row>
     <row r="25" ht="43.2" customHeight="1"/>
     <row r="26" ht="28.8" customHeight="1"/>
     <row r="27" ht="28.8" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 02 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -1944,7 +1944,60 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="43.2" customHeight="1"/>
+    <row r="25" ht="43.2" customHeight="1">
+      <c r="A25" s="13" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B25" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C25" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D25" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="E25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G25" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H25" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I25" s="15">
+        <f>IF(SUM(B25:F25,H25)=0,"",SUM(B25:F25,H25))</f>
+        <v/>
+      </c>
+      <c r="J25" s="15">
+        <f>IF(I25="","",1440-I25)</f>
+        <v/>
+      </c>
+      <c r="K25" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L25" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M25" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N25" s="17" t="inlineStr">
+        <is>
+          <t>Classes were a little tiring and did some revision after coming home.</t>
+        </is>
+      </c>
+    </row>
     <row r="26" ht="28.8" customHeight="1"/>
     <row r="27" ht="28.8" customHeight="1"/>
     <row r="28" ht="28.8" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 03 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -1998,7 +1998,60 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="28.8" customHeight="1"/>
+    <row r="26" ht="28.8" customHeight="1">
+      <c r="A26" s="13" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B26" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C26" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="D26" s="14" t="n">
+        <v>240</v>
+      </c>
+      <c r="E26" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G26" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H26" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="I26" s="15">
+        <f>IF(SUM(B26:F26,H26)=0,"",SUM(B26:F26,H26))</f>
+        <v/>
+      </c>
+      <c r="J26" s="15">
+        <f>IF(I26="","",1440-I26)</f>
+        <v/>
+      </c>
+      <c r="K26" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L26" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M26" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N26" s="17" t="inlineStr">
+        <is>
+          <t>Had regular classes and preparing for CA1 at home.</t>
+        </is>
+      </c>
+    </row>
     <row r="27" ht="28.8" customHeight="1"/>
     <row r="28" ht="28.8" customHeight="1"/>
     <row r="29" ht="28.8" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 04 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -2052,7 +2052,60 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="28.8" customHeight="1"/>
+    <row r="27" ht="28.8" customHeight="1">
+      <c r="A27" s="13" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B27" s="14" t="n">
+        <v>360</v>
+      </c>
+      <c r="C27" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="D27" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="E27" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F27" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H27" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I27" s="15">
+        <f>IF(SUM(B27:F27,H27)=0,"",SUM(B27:F27,H27))</f>
+        <v/>
+      </c>
+      <c r="J27" s="15">
+        <f>IF(I27="","",1440-I27)</f>
+        <v/>
+      </c>
+      <c r="K27" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L27" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M27" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N27" s="17" t="inlineStr">
+        <is>
+          <t>Had regular classes and preparing for CA1 at home.</t>
+        </is>
+      </c>
+    </row>
     <row r="28" ht="28.8" customHeight="1"/>
     <row r="29" ht="28.8" customHeight="1"/>
     <row r="30" ht="43.2" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 05 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -2106,7 +2106,60 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="28.8" customHeight="1"/>
+    <row r="28" ht="28.8" customHeight="1">
+      <c r="A28" s="13" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B28" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="E28" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I28" s="15">
+        <f>IF(SUM(B28:F28,H28)=0,"",SUM(B28:F28,H28))</f>
+        <v/>
+      </c>
+      <c r="J28" s="15">
+        <f>IF(I28="","",1440-I28)</f>
+        <v/>
+      </c>
+      <c r="K28" s="16" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L28" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M28" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N28" s="17" t="inlineStr">
+        <is>
+          <t>No regular classes. Preparing for CA1 at home and relaxed.</t>
+        </is>
+      </c>
+    </row>
     <row r="29" ht="28.8" customHeight="1"/>
     <row r="30" ht="43.2" customHeight="1"/>
     <row r="31" ht="43.2" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 06 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -2160,7 +2160,60 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="28.8" customHeight="1"/>
+    <row r="29" ht="28.8" customHeight="1">
+      <c r="A29" s="13" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B29" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="C29" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="E29" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="I29" s="15">
+        <f>IF(SUM(B29:F29,H29)=0,"",SUM(B29:F29,H29))</f>
+        <v/>
+      </c>
+      <c r="J29" s="15">
+        <f>IF(I29="","",1440-I29)</f>
+        <v/>
+      </c>
+      <c r="K29" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L29" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M29" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N29" s="17" t="inlineStr">
+        <is>
+          <t>No regular classes. Preparing for CA1 at home and relaxed.</t>
+        </is>
+      </c>
+    </row>
     <row r="30" ht="43.2" customHeight="1"/>
     <row r="31" ht="43.2" customHeight="1"/>
     <row r="34" ht="28.8" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 07 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -2214,7 +2214,60 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="43.2" customHeight="1"/>
+    <row r="30" ht="43.2" customHeight="1">
+      <c r="A30" s="13" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B30" s="14" t="n">
+        <v>240</v>
+      </c>
+      <c r="C30" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D30" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="E30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="G30" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H30" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I30" s="15">
+        <f>IF(SUM(B30:F30,H30)=0,"",SUM(B30:F30,H30))</f>
+        <v/>
+      </c>
+      <c r="J30" s="15">
+        <f>IF(I30="","",1440-I30)</f>
+        <v/>
+      </c>
+      <c r="K30" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L30" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M30" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N30" s="17" t="inlineStr">
+        <is>
+          <t>Had a CA today. Attended classes and revised the important topics at home.</t>
+        </is>
+      </c>
+    </row>
     <row r="31" ht="43.2" customHeight="1"/>
     <row r="34" ht="28.8" customHeight="1"/>
     <row r="35" ht="43.2" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 08 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -2268,7 +2268,60 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="43.2" customHeight="1"/>
+    <row r="31" ht="43.2" customHeight="1">
+      <c r="A31" s="13" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B31" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="C31" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="D31" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="E31" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="F31" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G31" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H31" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I31" s="15">
+        <f>IF(SUM(B31:F31,H31)=0,"",SUM(B31:F31,H31))</f>
+        <v/>
+      </c>
+      <c r="J31" s="15">
+        <f>IF(I31="","",1440-I31)</f>
+        <v/>
+      </c>
+      <c r="K31" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L31" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M31" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N31" s="17" t="inlineStr">
+        <is>
+          <t>Had regular classes and preparing for DBMS CA1 at home.</t>
+        </is>
+      </c>
+    </row>
     <row r="34" ht="28.8" customHeight="1"/>
     <row r="35" ht="43.2" customHeight="1"/>
     <row r="36" ht="43.2" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 09 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -2319,6 +2319,60 @@
       <c r="N31" s="17" t="inlineStr">
         <is>
           <t>Had regular classes and preparing for DBMS CA1 at home.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B32" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="C32" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="D32" s="14" t="n">
+        <v>360</v>
+      </c>
+      <c r="E32" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G32" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H32" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I32" s="15">
+        <f>IF(SUM(B32:F32,H32)=0,"",SUM(B32:F32,H32))</f>
+        <v/>
+      </c>
+      <c r="J32" s="15">
+        <f>IF(I32="","",1440-I32)</f>
+        <v/>
+      </c>
+      <c r="K32" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L32" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M32" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N32" s="17" t="inlineStr">
+        <is>
+          <t>Had regular classes.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 10 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N32"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -2373,6 +2373,60 @@
       <c r="N32" s="17" t="inlineStr">
         <is>
           <t>Had regular classes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B33" s="14" t="n">
+        <v>240</v>
+      </c>
+      <c r="C33" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="D33" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E33" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="14" t="n">
+        <v>90</v>
+      </c>
+      <c r="I33" s="15">
+        <f>IF(SUM(B33:F33,H33)=0,"",SUM(B33:F33,H33))</f>
+        <v/>
+      </c>
+      <c r="J33" s="15">
+        <f>IF(I33="","",1440-I33)</f>
+        <v/>
+      </c>
+      <c r="K33" s="16" t="inlineStr">
+        <is>
+          <t>Stressed</t>
+        </is>
+      </c>
+      <c r="L33" s="16" t="inlineStr">
+        <is>
+          <t>Very Unsatisfied</t>
+        </is>
+      </c>
+      <c r="M33" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N33" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Attend Fresher's Party. </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 11 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N33"/>
+  <dimension ref="A1:N34"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -2430,7 +2430,60 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="28.8" customHeight="1"/>
+    <row r="34" ht="28.8" customHeight="1">
+      <c r="A34" s="13" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B34" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C34" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="D34" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="E34" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="G34" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H34" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I34" s="15">
+        <f>IF(SUM(B34:F34,H34)=0,"",SUM(B34:F34,H34))</f>
+        <v/>
+      </c>
+      <c r="J34" s="15">
+        <f>IF(I34="","",1440-I34)</f>
+        <v/>
+      </c>
+      <c r="K34" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L34" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M34" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N34" s="17" t="inlineStr">
+        <is>
+          <t>Had regular classes and completed a little study at night.</t>
+        </is>
+      </c>
+    </row>
     <row r="35" ht="43.2" customHeight="1"/>
     <row r="36" ht="43.2" customHeight="1"/>
     <row r="37" ht="28.8" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 12 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -2484,7 +2484,60 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="43.2" customHeight="1"/>
+    <row r="35" ht="43.2" customHeight="1">
+      <c r="A35" s="13" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B35" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C35" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D35" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E35" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="I35" s="15">
+        <f>IF(SUM(B35:F35,H35)=0,"",SUM(B35:F35,H35))</f>
+        <v/>
+      </c>
+      <c r="J35" s="15">
+        <f>IF(I35="","",1440-I35)</f>
+        <v/>
+      </c>
+      <c r="K35" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L35" s="16" t="inlineStr">
+        <is>
+          <t>Unsatisfied</t>
+        </is>
+      </c>
+      <c r="M35" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N35" s="17" t="inlineStr">
+        <is>
+          <t>No classes today. Studied at home, watched movie and relaxed.</t>
+        </is>
+      </c>
+    </row>
     <row r="36" ht="43.2" customHeight="1"/>
     <row r="37" ht="28.8" customHeight="1"/>
     <row r="38" ht="28.8" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 13 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:N36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -2538,7 +2538,60 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="43.2" customHeight="1"/>
+    <row r="36" ht="43.2" customHeight="1">
+      <c r="A36" s="13" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B36" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C36" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="D36" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="E36" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="I36" s="15">
+        <f>IF(SUM(B36:F36,H36)=0,"",SUM(B36:F36,H36))</f>
+        <v/>
+      </c>
+      <c r="J36" s="15">
+        <f>IF(I36="","",1440-I36)</f>
+        <v/>
+      </c>
+      <c r="K36" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L36" s="16" t="inlineStr">
+        <is>
+          <t>Very Satisfied</t>
+        </is>
+      </c>
+      <c r="M36" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N36" s="17" t="inlineStr">
+        <is>
+          <t>No classes today. Studied at home, watched movie and relaxed.</t>
+        </is>
+      </c>
+    </row>
     <row r="37" ht="28.8" customHeight="1"/>
     <row r="38" ht="28.8" customHeight="1"/>
     <row r="39" ht="43.2" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 14 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:N37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -2592,7 +2592,60 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="28.8" customHeight="1"/>
+    <row r="37" ht="28.8" customHeight="1">
+      <c r="A37" s="13" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B37" s="14" t="n">
+        <v>360</v>
+      </c>
+      <c r="C37" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D37" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E37" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="G37" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H37" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I37" s="15">
+        <f>IF(SUM(B37:F37,H37)=0,"",SUM(B37:F37,H37))</f>
+        <v/>
+      </c>
+      <c r="J37" s="15">
+        <f>IF(I37="","",1440-I37)</f>
+        <v/>
+      </c>
+      <c r="K37" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L37" s="16" t="inlineStr">
+        <is>
+          <t>Unsatisfied</t>
+        </is>
+      </c>
+      <c r="M37" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N37" s="17" t="inlineStr">
+        <is>
+          <t>Had classes and preparing for Python CA1 at home.</t>
+        </is>
+      </c>
+    </row>
     <row r="38" ht="28.8" customHeight="1"/>
     <row r="39" ht="43.2" customHeight="1"/>
     <row r="40" ht="43.2" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 15 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N37"/>
+  <dimension ref="A1:N38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -2646,7 +2646,60 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="28.8" customHeight="1"/>
+    <row r="38" ht="28.8" customHeight="1">
+      <c r="A38" s="13" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B38" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C38" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D38" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E38" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G38" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H38" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="I38" s="15">
+        <f>IF(SUM(B38:F38,H38)=0,"",SUM(B38:F38,H38))</f>
+        <v/>
+      </c>
+      <c r="J38" s="15">
+        <f>IF(I38="","",1440-I38)</f>
+        <v/>
+      </c>
+      <c r="K38" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L38" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M38" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N38" s="17" t="inlineStr">
+        <is>
+          <t>Had classes and give Python CA1 at home through Online.</t>
+        </is>
+      </c>
+    </row>
     <row r="39" ht="43.2" customHeight="1"/>
     <row r="40" ht="43.2" customHeight="1"/>
     <row r="41" ht="43.2" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 16 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N38"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -2700,7 +2700,60 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="43.2" customHeight="1"/>
+    <row r="39" ht="43.2" customHeight="1">
+      <c r="A39" s="13" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B39" s="14" t="n">
+        <v>540</v>
+      </c>
+      <c r="C39" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D39" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E39" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="G39" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H39" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I39" s="15">
+        <f>IF(SUM(B39:F39,H39)=0,"",SUM(B39:F39,H39))</f>
+        <v/>
+      </c>
+      <c r="J39" s="15">
+        <f>IF(I39="","",1440-I39)</f>
+        <v/>
+      </c>
+      <c r="K39" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L39" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M39" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N39" s="17" t="inlineStr">
+        <is>
+          <t>Had classes and some classes was exempted and solving maths at home.</t>
+        </is>
+      </c>
+    </row>
     <row r="40" ht="43.2" customHeight="1"/>
     <row r="41" ht="43.2" customHeight="1"/>
     <row r="42" ht="43.2" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 17 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N39"/>
+  <dimension ref="A1:N40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -2754,7 +2754,60 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="43.2" customHeight="1"/>
+    <row r="40" ht="43.2" customHeight="1">
+      <c r="A40" s="13" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B40" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C40" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D40" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="E40" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F40" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G40" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H40" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I40" s="15">
+        <f>IF(SUM(B40:F40,H40)=0,"",SUM(B40:F40,H40))</f>
+        <v/>
+      </c>
+      <c r="J40" s="15">
+        <f>IF(I40="","",1440-I40)</f>
+        <v/>
+      </c>
+      <c r="K40" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L40" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M40" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N40" s="17" t="inlineStr">
+        <is>
+          <t>Had regular classes and preparing  for Analytical skill CA1 at night.</t>
+        </is>
+      </c>
+    </row>
     <row r="41" ht="43.2" customHeight="1"/>
     <row r="42" ht="43.2" customHeight="1"/>
     <row r="43" ht="43.2" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 18 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N40"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -2808,7 +2808,60 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="43.2" customHeight="1"/>
+    <row r="41" ht="43.2" customHeight="1">
+      <c r="A41" s="13" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B41" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C41" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D41" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="E41" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F41" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G41" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H41" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I41" s="15">
+        <f>IF(SUM(B41:F41,H41)=0,"",SUM(B41:F41,H41))</f>
+        <v/>
+      </c>
+      <c r="J41" s="15">
+        <f>IF(I41="","",1440-I41)</f>
+        <v/>
+      </c>
+      <c r="K41" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L41" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M41" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N41" s="17" t="inlineStr">
+        <is>
+          <t>Had regular classes and preparing  for Analytical skill CA1 at night.</t>
+        </is>
+      </c>
+    </row>
     <row r="42" ht="43.2" customHeight="1"/>
     <row r="43" ht="43.2" customHeight="1"/>
     <row r="44" ht="43.2" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 19 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -2862,7 +2862,60 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="43.2" customHeight="1"/>
+    <row r="42" ht="43.2" customHeight="1">
+      <c r="A42" s="13" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B42" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C42" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="D42" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E42" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="14" t="n">
+        <v>90</v>
+      </c>
+      <c r="I42" s="15">
+        <f>IF(SUM(B42:F42,H42)=0,"",SUM(B42:F42,H42))</f>
+        <v/>
+      </c>
+      <c r="J42" s="15">
+        <f>IF(I42="","",1440-I42)</f>
+        <v/>
+      </c>
+      <c r="K42" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L42" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M42" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N42" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No classes today. Had an Analytical Skills test, and overall it was a good day. </t>
+        </is>
+      </c>
+    </row>
     <row r="43" ht="43.2" customHeight="1"/>
     <row r="44" ht="43.2" customHeight="1"/>
     <row r="45" ht="43.2" customHeight="1"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 20 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N42"/>
+  <dimension ref="A1:N43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -2916,7 +2916,60 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="43.2" customHeight="1"/>
+    <row r="43" ht="43.2" customHeight="1">
+      <c r="A43" s="13" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B43" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C43" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="D43" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="E43" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="F43" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="I43" s="15">
+        <f>IF(SUM(B43:F43,H43)=0,"",SUM(B43:F43,H43))</f>
+        <v/>
+      </c>
+      <c r="J43" s="15">
+        <f>IF(I43="","",1440-I43)</f>
+        <v/>
+      </c>
+      <c r="K43" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L43" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M43" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N43" s="17" t="inlineStr">
+        <is>
+          <t>Preparing for English Communication CA2 at home, watched movie and relaxed.</t>
+        </is>
+      </c>
+    </row>
     <row r="44" ht="43.2" customHeight="1"/>
     <row r="45" ht="43.2" customHeight="1"/>
   </sheetData>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 21 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N43"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -2970,7 +2970,60 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="43.2" customHeight="1"/>
+    <row r="44" ht="43.2" customHeight="1">
+      <c r="A44" s="13" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B44" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C44" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="D44" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="E44" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="G44" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H44" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="I44" s="15">
+        <f>IF(SUM(B44:F44,H44)=0,"",SUM(B44:F44,H44))</f>
+        <v/>
+      </c>
+      <c r="J44" s="15">
+        <f>IF(I44="","",1440-I44)</f>
+        <v/>
+      </c>
+      <c r="K44" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L44" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M44" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N44" s="17" t="inlineStr">
+        <is>
+          <t>Attended classes and revised the important topics of DBMS at home.</t>
+        </is>
+      </c>
+    </row>
     <row r="45" ht="43.2" customHeight="1"/>
   </sheetData>
   <mergeCells count="6">

</xml_diff>

<commit_message>
Update 12626434.xlsx - 22 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -3024,7 +3024,60 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="43.2" customHeight="1"/>
+    <row r="45" ht="43.2" customHeight="1">
+      <c r="A45" s="13" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B45" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C45" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="D45" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="E45" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="F45" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G45" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H45" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I45" s="15">
+        <f>IF(SUM(B45:F45,H45)=0,"",SUM(B45:F45,H45))</f>
+        <v/>
+      </c>
+      <c r="J45" s="15">
+        <f>IF(I45="","",1440-I45)</f>
+        <v/>
+      </c>
+      <c r="K45" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L45" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M45" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N45" s="17" t="inlineStr">
+        <is>
+          <t>Had regular classes and preparing  for DBMS CA2 at night.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="F3:G3"/>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 23 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N45"/>
+  <dimension ref="A1:N46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -3075,6 +3075,60 @@
       <c r="N45" s="17" t="inlineStr">
         <is>
           <t>Had regular classes and preparing  for DBMS CA2 at night.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="13" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B46" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C46" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D46" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E46" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G46" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H46" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="I46" s="15">
+        <f>IF(SUM(B46:F46,H46)=0,"",SUM(B46:F46,H46))</f>
+        <v/>
+      </c>
+      <c r="J46" s="15">
+        <f>IF(I46="","",1440-I46)</f>
+        <v/>
+      </c>
+      <c r="K46" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L46" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M46" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N46" s="17" t="inlineStr">
+        <is>
+          <t>Had classes and give DBMS CA2.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 12626434.xlsx - 25 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ANISH\OneDrive\Documents\GitHub\python_minor_project_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E5CEF8-C667-46BE-8E77-599C10AA7FBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE51E84C-599F-4965-9339-C316FF9AB804}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="14016" windowHeight="12336" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2652" yWindow="2652" windowWidth="17280" windowHeight="8880" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="93">
   <si>
     <t>My Data, My Code — Daily Log</t>
   </si>
@@ -310,6 +310,9 @@
   </si>
   <si>
     <t>Watching movie.</t>
+  </si>
+  <si>
+    <t>Had regular classes and preparing  for English communications CA2 at night.</t>
   </si>
 </sst>
 </file>
@@ -523,19 +526,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1167,7 +1158,7 @@
         <v>30</v>
       </c>
       <c r="I6" s="10">
-        <f t="shared" ref="I6:I47" si="0">IF(SUM(B6:F6,H6)=0,"",SUM(B6:F6,H6))</f>
+        <f t="shared" ref="I6:I48" si="0">IF(SUM(B6:F6,H6)=0,"",SUM(B6:F6,H6))</f>
         <v>885</v>
       </c>
       <c r="J6" s="10">
@@ -3073,27 +3064,51 @@
         <v>91</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A48" s="13"/>
-      <c r="B48" s="14"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
-      <c r="F48" s="14"/>
-      <c r="G48" s="14"/>
-      <c r="H48" s="14"/>
-      <c r="I48" s="15" t="str">
-        <f t="shared" ref="I47:I110" si="2">IF(SUM(B48:F48,H48)=0,"",SUM(B48:F48,H48))</f>
-        <v/>
-      </c>
-      <c r="J48" s="15" t="str">
+    <row r="48" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A48" s="13">
+        <v>46290</v>
+      </c>
+      <c r="B48" s="14">
+        <v>480</v>
+      </c>
+      <c r="C48" s="14">
+        <v>60</v>
+      </c>
+      <c r="D48" s="14">
+        <v>120</v>
+      </c>
+      <c r="E48" s="14">
+        <v>0</v>
+      </c>
+      <c r="F48" s="14">
+        <v>300</v>
+      </c>
+      <c r="G48" s="14">
+        <v>6</v>
+      </c>
+      <c r="H48" s="14">
+        <v>90</v>
+      </c>
+      <c r="I48" s="15">
+        <f t="shared" si="0"/>
+        <v>1050</v>
+      </c>
+      <c r="J48" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K48" s="14"/>
-      <c r="L48" s="14"/>
-      <c r="M48" s="14"/>
-      <c r="N48" s="14"/>
+        <v>390</v>
+      </c>
+      <c r="K48" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="L48" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="M48" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="N48" s="17" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" s="13"/>
@@ -3105,7 +3120,7 @@
       <c r="G49" s="14"/>
       <c r="H49" s="14"/>
       <c r="I49" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="I48:I110" si="2">IF(SUM(B49:F49,H49)=0,"",SUM(B49:F49,H49))</f>
         <v/>
       </c>
       <c r="J49" s="15" t="str">
@@ -6426,26 +6441,26 @@
     <mergeCell ref="A4:N4"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>
-  <conditionalFormatting sqref="J6:J46 J48:J230">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="lessThan">
+  <conditionalFormatting sqref="J6:J47 J49:J230">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J47">
+  <conditionalFormatting sqref="J48">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" error="Please choose a value from the dropdown list." prompt="Select today's overall feeling" sqref="K6:K47 K200:K230" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" error="Please choose a value from the dropdown list." prompt="Select today's overall feeling" sqref="K6:K48 K200:K230" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Excellent,Good,Neutral,Low,Stressed"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" prompt="Select today's satisfaction level" sqref="L6:L47 L200:L230" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" prompt="Select today's satisfaction level" sqref="L6:L48 L200:L230" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Very Satisfied,Satisfied,Neutral,Unsatisfied,Very Unsatisfied"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" prompt="Select today's energy level" sqref="M6:M47 M200:M230" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" allowBlank="1" prompt="Select today's energy level" sqref="M6:M48 M200:M230" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"High,Medium,Low"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>